<commit_message>
feat: one subfolder per mos-geo skill, brand-audit-master.xlsx at the month root
campaigns/geo/YYYY-MM/{brand-audit-master.xlsx, brand-360-report/, llm-buttons/}.
brand360.py path/workbook follow the new shape; tick_checklist.py lets any
skill mark its Checklist row; mos-geo-llm-buttons writes into llm-buttons/.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KvgWPsLwwubaVx79jaEZ5B
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/brand-360-report.md (agency HQ: campaigns/geo/YYYY-MM/&lt;brand&gt;/)</t>
+          <t>campaigns/geo/YYYY-MM/brand-360-report/</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/llm-buttons/ (see the skill)</t>
+          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat(mos-geo-ai-info): AI Info Page skill + brand audit integration
New skill: crawl the brand's site, write sourced data/facts.json, and let
aiinfo.py build render the page (md + html with Organization JSON-LD),
ai-info.json and a developer handover, lint every statement for a source,
then add an 'AI Info Page' approval tab, Checklist tick and publish task to
brand-audit-master.xlsx. check tests the live page. Canary line is opt-in.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QaEJ9y9nZ9asgknNK5RZvX
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -662,32 +662,32 @@
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Content Strategy</t>
+          <t>Brand Optimisation</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-llm-buttons</t>
+          <t>mos-geo-ai-info</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
+          <t>AI Info Page: an official, sourced fact sheet for ChatGPT, Claude, Perplexity and Gemini (basic info, background, services, clients, methods, advantages, guidance for AI), with schema, a machine-readable JSON copy and a developer handover.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-llm-buttons</t>
+          <t>/mos-geo-ai-info</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
+          <t>campaigns/geo/YYYY-MM/ai-info/</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>AI Info Page, Initiatives</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -704,23 +704,51 @@
       <c r="K9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="n"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Content Strategy</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-llm-buttons</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-llm-buttons</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Initiatives</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="n"/>
       <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-llm-buttons: Client website URL</t>
-        </is>
-      </c>
+      <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
@@ -732,7 +760,11 @@
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="4" t="n"/>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL</t>
+        </is>
+      </c>
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
@@ -1421,6 +1453,7 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(mos-geo-google-preferred-sources): new skill for Google's preferred-source button
Checks eligibility, stack and CSP; builds a button in the site's own style from
Google's documented manual-mode code with a deeplink fallback; places it after the
strongest paragraph; installs directly or writes a developer handover; verifies the
live install with a stdlib script (45 tests). Registered in README, skills.json,
the audit workbook template and geo-evidence.md section 9.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5xfgbvLy1LKKnvzqeUh7F
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -968,23 +968,51 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Brand Optimisation</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-google-preferred-sources</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Google 'Add as a preferred source' button: eligibility check, a button styled to the site using Google's official code, placement after the best paragraph, and a live verify. Readers who choose the site see it more in Top Stories and get a 'preferred' badge in AI Overviews and AI Mode.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-google-preferred-sources</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/preferred-sources/</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Initiatives</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="n"/>
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-dealbreakers: Client website URL (community or marketplace URLs optional); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+; mos-geo-fan-out-map: Gemini API key (free tier)</t>
-        </is>
-      </c>
+      <c r="B17" s="4" t="n"/>
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
@@ -996,7 +1024,11 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="4" t="n"/>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-dealbreakers: Client website URL (community or marketplace URLs optional); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+; mos-geo-fan-out-map: Gemini API key (free tier); mos-geo-google-preferred-sources: Client website URL (site code or WordPress access to install; otherwise a developer handover)</t>
+        </is>
+      </c>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
@@ -1619,6 +1651,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(mos-geo-schema-scraper): read JSON-LD from a Screaming Frog crawl, Apify opt-in
The scraper now reads schema for free from Screaming Frog instead of spending
Apify credits:

- --sf-csv: Custom Extraction export (Address + every JSON-LD n column),
  non-200 / non-HTML / non-indexable rows skipped and reported
- --sf-html: stored page source, mapped to URLs like mos-geo-internal-links
  (canonical, og:url, file name; rendered_ copies preferred)
- each script becomes one block; comment/CDATA wrappers stripped; empty -> {};
  invalid JSON kept as {"_unparsed": ...} and flagged
- --url/--urls filter a crawl; run record in raw/_sf-runs/
- Apify kept behind --source apify (--country only there)

SKILL.md rewritten around one shared crawl; README, skills.json and the
workbook template updated; the optimisation skill points at the same crawl.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XmciGqvh3Dde6iWgRRyNj1
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -804,7 +804,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Live JSON-LD snapshot of a URL list, rendered in a real browser so tag-manager and JavaScript schema is caught: one pure-JSON file per page ([] if none), sorted by page type. The 'before' state for a schema rebuild.</t>
+          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -894,7 +894,7 @@
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Apify token (APIFY_TOKEN or `apify login`), a URL list; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV); Node 18+</t>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
         </is>
       </c>
       <c r="C15" s="4" t="n"/>

</xml_diff>

<commit_message>
feat(mos-geo-fan-out): page-level query fan-out and citability audit
New skill: for 1 to 500+ pages, drafts buyer prompts per page, pulls the
searches ChatGPT runs for them (DataForSEO LLM Responses fan_out_queries,
repeated runs for stability), classifies each (site: vendor, exact string,
open), checks page coverage and optional SERP retrieval, records the
citation baseline, and writes a site report, per-page fix lists and a
Fan-Out tab in the brand audit workbook. Resumable raw cache, hard spend
cap, retest for measuring lift. Default model gpt-5.6-luna (~$0.024/call).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017dhx4CBy6hpQJbtGEMfxtz
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -748,31 +748,91 @@
       <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="n"/>
-      <c r="I11" s="4" t="n"/>
-      <c r="J11" s="4" t="n"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Technical Foundations</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-internal-links</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-internal-links</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>None yet (audit and recommendations live in the run folder)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="n"/>
       <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Content Strategy</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-fan-out</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>For 1 to 500+ pages, finds the searches AI engines actually run (query fan-out) for the prompts each page should win, measures whether the page is cited today, and produces a per-page fix list (add exact string, add section, earn retrieval, skip unwinnable vendor searches) ranked by stability.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-fan-out</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/fan-out/</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Fan-Out, Initiatives</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="n"/>
       <c r="K12" s="4" t="n"/>
     </row>
     <row r="13">
@@ -788,7 +848,11 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="n"/>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-fan-out: DataForSEO (LLM Responses + LLM Mentions)</t>
+        </is>
+      </c>
       <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="n"/>
@@ -1454,6 +1518,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: rename mos-geo-fan-out to mos-geo-query-fan-out
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JsGP2fZNg7XBb7Jy6MTnB6
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K67"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -535,6 +535,7 @@
     <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -563,6 +564,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -799,7 +801,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-fan-out</t>
+          <t>mos-geo-query-fan-out</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -809,7 +811,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-fan-out</t>
+          <t>/mos-geo-query-fan-out</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -850,7 +852,7 @@
     <row r="14">
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-fan-out: DataForSEO (LLM Responses + LLM Mentions)</t>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-query-fan-out: DataForSEO (LLM Responses + LLM Mentions)</t>
         </is>
       </c>
       <c r="C14" s="4" t="n"/>
@@ -1531,7 +1533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J67"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1546,6 +1548,7 @@
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1574,6 +1577,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="32" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -2513,7 +2517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:M65"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2531,6 +2535,7 @@
     <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2545,6 +2550,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add mos-geo-dealbreakers (Dealbreaker Detector)
Crawl buying pages plus an off-site sweep, typed evidence (stated,
contradicted, absent, inferred), a build step that verifies every quote
against saved page text, then renders the report, FAQ draft and CSV and
fills a Dealbreakers tab plus Initiatives in the brand audit workbook.
Method credited to Steve Toth (Notebook Agency); independent implementation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQryY74faMbumjwomkKevY
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brand Truth Review" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Truth Review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$B$7:$K$67</definedName>
@@ -711,27 +711,27 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-llm-buttons</t>
+          <t>mos-geo-dealbreakers</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
+          <t>Dealbreaker Detector: reads the brand's public site, community and reviews as a sceptical buyer and lists every reason a qualified buyer would walk away (proof, pricing, setup, maturity, risk, fit), each with a verified quote or the pages checked, plus priorities, what's already handled and an FAQ draft.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-llm-buttons</t>
+          <t>/mos-geo-dealbreakers</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
+          <t>campaigns/geo/YYYY-MM/dealbreakers/</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>Dealbreakers, Initiatives</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -750,32 +750,32 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Technical Foundations</t>
+          <t>Content Strategy</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-internal-links</t>
+          <t>mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
+          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-internal-links</t>
+          <t>/mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
+          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>None yet (audit and recommendations live in the run folder)</t>
+          <t>Initiatives</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -799,27 +799,27 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-scraper</t>
+          <t>mos-geo-internal-links</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
+          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-scraper</t>
+          <t>/mos-geo-internal-links</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/schema/</t>
+          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>None yet (outputs live in the schema folder)</t>
+          <t>None yet (audit and recommendations live in the run folder)</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-optimisation</t>
+          <t>mos-geo-schema-scraper</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
+          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-optimisation</t>
+          <t>/mos-geo-schema-scraper</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -880,23 +880,51 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Technical Foundations</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-schema-optimisation</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-schema-optimisation</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/schema/</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>None yet (outputs live in the schema folder)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="n"/>
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
-        </is>
-      </c>
+      <c r="B15" s="4" t="n"/>
       <c r="C15" s="4" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
@@ -908,7 +936,11 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="n"/>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-dealbreakers: Client website URL (community or marketplace URLs optional); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
+        </is>
+      </c>
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
@@ -1553,6 +1585,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: sync pending work (19 files, 2026-10-01)
- mos-geo-topic-clusters (5 files)
- mos-geo-ai-info-generator (5 files)
- .claude (5 files)
- _shared (2 files)
- mos-geo-ai-info (1 files)
- README.md (1 files)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WKJTouaCqwfP4jpmxUnDfd
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -706,32 +706,32 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Content Strategy</t>
+          <t>Brand Optimisation</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-llm-buttons</t>
+          <t>mos-geo-ai-info-generator</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
+          <t>Fast AI Info Page draft in the exact shape of Steve Toth's GPT, written from the brand's own brain, site crawl and a short interview; a lint gate fails any missing section or any number not in those inputs.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-llm-buttons</t>
+          <t>/mos-geo-ai-info-generator</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
+          <t>campaigns/geo/YYYY-MM/ai-info-draft/</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>None yet (page.md, page.html and handover.md live in the run folder)</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -750,32 +750,32 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Technical Foundations</t>
+          <t>Brand Optimisation</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-internal-links</t>
+          <t>mos-geo-homepage-faqs</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
+          <t>12 to 20 homepage FAQs written for AI assistants to quote: one self-contained sentence per answer, entity first, every fact from the brand's own site, each linked to the internal page that backs it up, with FAQPage schema and a client approval tab.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-internal-links</t>
+          <t>/mos-geo-homepage-faqs</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
+          <t>campaigns/geo/YYYY-MM/homepage-faqs/</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>None yet (audit and recommendations live in the run folder)</t>
+          <t>Homepage FAQs, Initiatives</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -794,32 +794,32 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Technical Foundations</t>
+          <t>Content Strategy</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-scraper</t>
+          <t>mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
+          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-scraper</t>
+          <t>/mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/schema/</t>
+          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>None yet (outputs live in the schema folder)</t>
+          <t>Initiatives</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -843,27 +843,27 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-optimisation</t>
+          <t>mos-geo-internal-links</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
+          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-optimisation</t>
+          <t>/mos-geo-internal-links</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/schema/</t>
+          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>None yet (outputs live in the schema folder)</t>
+          <t>None yet (audit and recommendations live in the run folder)</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -880,43 +880,135 @@
       <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Content Strategy</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-topic-clusters</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Keyword clusters (one cluster = one page) rolled up into topics with a pillar, each mapped to the page ranking today, with status (Owned, Striking, Cannibalised, Lost ...), opportunity score, home-page overload and a cannibalisation list; pairs judged by TypeSafe Jev, clusters and numbers built in code.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-topic-clusters</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/mos-geo-topic-clusters/</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>None yet (xlsx and README live in the run folder)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="n"/>
       <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-      <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Technical Foundations</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-schema-scraper</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-schema-scraper</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/schema/</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>None yet (outputs live in the schema folder)</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="n"/>
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Technical Foundations</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-schema-optimisation</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-schema-optimisation</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/schema/</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>None yet (outputs live in the schema folder)</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="n"/>
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
@@ -932,7 +1024,11 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="4" t="n"/>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-ai-info-generator: Brand website URL; a MarketingOS brain if there is one; mos-geo-homepage-faqs: Brand name and website URL; Scrapling recommended (uses AI Info Page and Brand 360 outputs when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-topic-clusters: Ahrefs Organic Keywords export or GSC page+query export; TypeSafe API key; OpenAI or Voyage key optional (embeddings); DataForSEO optional (SERP overlap); mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
+        </is>
+      </c>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
@@ -1553,6 +1649,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve homepage FAQ skill evidence review and export validation
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Brand Truth Review" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand Truth Review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$B$7:$K$67</definedName>
@@ -711,27 +711,27 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-ai-info-generator</t>
+          <t>mos-geo-homepage-faqs</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Fast AI Info Page draft in the exact shape of Steve Toth's GPT, written from the brand's own brain, site crawl and a short interview; a lint gate fails any missing section or any number not in those inputs.</t>
+          <t>Sourced, entity-first FAQs ranked for a homepage and FAQ page, with passage-level claim review, verified internal links where useful, matching FAQPage schema and a client approval tab; exports require current final lint.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-ai-info-generator</t>
+          <t>/mos-geo-homepage-faqs</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/ai-info-draft/</t>
+          <t>campaigns/geo/YYYY-MM/homepage-faqs/</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>None yet (page.md, page.html and handover.md live in the run folder)</t>
+          <t>Homepage FAQs, Initiatives</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -750,32 +750,32 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Brand Optimisation</t>
+          <t>Content Strategy</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-homepage-faqs</t>
+          <t>mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>12 to 20 homepage FAQs written for AI assistants to quote: one self-contained sentence per answer, entity first, every fact from the brand's own site, each linked to the internal page that backs it up, with FAQPage schema and a client approval tab.</t>
+          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-homepage-faqs</t>
+          <t>/mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/homepage-faqs/</t>
+          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Homepage FAQs, Initiatives</t>
+          <t>Initiatives</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -794,32 +794,32 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Content Strategy</t>
+          <t>Technical Foundations</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-llm-buttons</t>
+          <t>mos-geo-internal-links</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
+          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-llm-buttons</t>
+          <t>/mos-geo-internal-links</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
+          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>None yet (audit and recommendations live in the run folder)</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -838,32 +838,32 @@
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Technical Foundations</t>
+          <t>Content Strategy</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-internal-links</t>
+          <t>mos-geo-topic-clusters</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
+          <t>Keyword clusters (one cluster = one page) rolled up into topics with a pillar, each mapped to the page ranking today, with status (Owned, Striking, Cannibalised, Lost ...), opportunity score, home-page overload and a cannibalisation list; pairs judged by TypeSafe Jev, clusters and numbers built in code.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-internal-links</t>
+          <t>/mos-geo-topic-clusters</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
+          <t>campaigns/geo/YYYY-MM/mos-geo-topic-clusters/</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>None yet (audit and recommendations live in the run folder)</t>
+          <t>None yet (xlsx and README live in the run folder)</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -882,32 +882,32 @@
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Content Strategy</t>
+          <t>Technical Foundations</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-topic-clusters</t>
+          <t>mos-geo-schema-scraper</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Keyword clusters (one cluster = one page) rolled up into topics with a pillar, each mapped to the page ranking today, with status (Owned, Striking, Cannibalised, Lost ...), opportunity score, home-page overload and a cannibalisation list; pairs judged by TypeSafe Jev, clusters and numbers built in code.</t>
+          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-topic-clusters</t>
+          <t>/mos-geo-schema-scraper</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/mos-geo-topic-clusters/</t>
+          <t>campaigns/geo/YYYY-MM/schema/</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>None yet (xlsx and README live in the run folder)</t>
+          <t>None yet (outputs live in the schema folder)</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -931,17 +931,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-scraper</t>
+          <t>mos-geo-schema-optimisation</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
+          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-scraper</t>
+          <t>/mos-geo-schema-optimisation</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -968,51 +968,23 @@
       <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Technical Foundations</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>mos-geo-schema-optimisation</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>/mos-geo-schema-optimisation</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>campaigns/geo/YYYY-MM/schema/</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>None yet (outputs live in the schema folder)</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="4" t="n"/>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-homepage-faqs: Brand name and website URL; Python 3.10+, openpyxl for the workbook; whole mos-geo-skills pack (Scrapling optional); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-topic-clusters: Ahrefs Organic Keywords export or GSC page+query export; TypeSafe API key; OpenAI or Voyage key optional (embeddings); DataForSEO optional (SERP overlap); mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
+        </is>
+      </c>
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
@@ -1024,11 +996,7 @@
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-ai-info-generator: Brand website URL; a MarketingOS brain if there is one; mos-geo-homepage-faqs: Brand name and website URL; Scrapling recommended (uses AI Info Page and Brand 360 outputs when present); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-topic-clusters: Ahrefs Organic Keywords export or GSC page+query export; TypeSafe API key; OpenAI or Voyage key optional (embeddings); DataForSEO optional (SERP overlap); mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+</t>
-        </is>
-      </c>
+      <c r="B18" s="4" t="n"/>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
@@ -1651,7 +1619,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(shared): register mos-geo-review-sentiment and add review-site evidence
Adds the skill to skills.json and rebuilds the audit template, adds a
README row, and adds geo-evidence section 11 (Semrush Nov 2025, Peec AI
Mar 2026) as the only basis for the skill's AI-citation claims.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FwxpAkNnR8vVFjMJg1YFBV
</commit_message>
<xml_diff>
--- a/_shared/brand-audit/brand-audit-template.xlsx
+++ b/_shared/brand-audit/brand-audit-template.xlsx
@@ -750,32 +750,32 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Content Strategy</t>
+          <t>Brand Optimisation</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-llm-buttons</t>
+          <t>mos-geo-review-sentiment</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
+          <t>Review sentiment audit: finds the brand's third-party review profiles (Trustpilot, Google Maps, ProductReview, G2, Capterra, Reddit and more), scrapes only the ones you pick, labels every review against an approved aspect taxonomy, and ranks the complaints to fix, with verbatim quotes, owners, a GEO action each, phrase word clouds and the unreplied 1 to 2 star reviews.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-llm-buttons</t>
+          <t>/mos-geo-review-sentiment</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
+          <t>campaigns/geo/YYYY-MM/review-sentiment/</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>Review Fixes, Initiatives</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -794,32 +794,32 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Technical Foundations</t>
+          <t>Content Strategy</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-internal-links</t>
+          <t>mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
+          <t>Client-ready LLM share buttons package: brief, code reference and an in-brand demo of 'ask ChatGPT / Claude / Perplexity about this page' buttons.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-internal-links</t>
+          <t>/mos-geo-llm-buttons</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
+          <t>campaigns/geo/YYYY-MM/llm-buttons/</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>None yet (audit and recommendations live in the run folder)</t>
+          <t>Initiatives</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -843,27 +843,27 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-scraper</t>
+          <t>mos-geo-internal-links</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
+          <t>Internal link audit (true contextual links vs template noise, orphans, deep pages, links to redirects and errors, anchor conflicts) plus reviewable contextual link recommendations: target, sentence and verbatim anchor, judged by TypeSafe Jev.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-scraper</t>
+          <t>/mos-geo-internal-links</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/schema/</t>
+          <t>campaigns/geo/YYYY-MM/mos-geo-internal-links/</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>None yet (outputs live in the schema folder)</t>
+          <t>None yet (audit and recommendations live in the run folder)</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -887,17 +887,17 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-schema-optimisation</t>
+          <t>mos-geo-schema-scraper</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
+          <t>Live JSON-LD snapshot of every page from a Screaming Frog crawl (custom extraction or stored HTML, JavaScript rendered): one pure-JSON file per page ([] if none), sorted by page type, broken blocks flagged. The 'before' state for a schema rebuild.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-schema-optimisation</t>
+          <t>/mos-geo-schema-scraper</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -926,32 +926,32 @@
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Content Strategy</t>
+          <t>Technical Foundations</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-fan-out-map</t>
+          <t>mos-geo-schema-optimisation</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Free, inventory-wide query fan-out. Predicts each page's query fan-out with Gemini Flash (no search, no spend) from a sitemap or URL list, scores each page's own coverage, and maps which pages to optimise and which topics across the inventory have no page. Predicted, not observed - confirm priority pages with a live ChatGPT / Google AI Mode check before writing or optimising.</t>
+          <t>Landscape Word brief: current schema audit plus the 3 to 5 highest-impact schemas, each with a developer template and an example filled with the brand's real values, unverified values raised as margin comments.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-fan-out-map</t>
+          <t>/mos-geo-schema-optimisation</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/mos-geo-fan-out-map/</t>
+          <t>campaigns/geo/YYYY-MM/schema/</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Fan-Out Map, Initiatives</t>
+          <t>None yet (outputs live in the schema folder)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -970,32 +970,32 @@
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Brand Optimisation</t>
+          <t>Content Strategy</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>mos-geo-google-preferred-sources</t>
+          <t>mos-geo-fan-out-map</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Google 'Add as a preferred source' button: eligibility check, a button styled to the site using Google's official code, placement after the best paragraph, and a live verify. Readers who choose the site see it more in Top Stories and get a 'preferred' badge in AI Overviews and AI Mode.</t>
+          <t>Free, inventory-wide query fan-out. Predicts each page's query fan-out with Gemini Flash (no search, no spend) from a sitemap or URL list, scores each page's own coverage, and maps which pages to optimise and which topics across the inventory have no page. Predicted, not observed - confirm priority pages with a live ChatGPT / Google AI Mode check before writing or optimising.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>/mos-geo-google-preferred-sources</t>
+          <t>/mos-geo-fan-out-map</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>campaigns/geo/YYYY-MM/preferred-sources/</t>
+          <t>campaigns/geo/YYYY-MM/mos-geo-fan-out-map/</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Initiatives</t>
+          <t>Fan-Out Map, Initiatives</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1012,23 +1012,51 @@
       <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="n"/>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Brand Optimisation</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>mos-geo-google-preferred-sources</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Google 'Add as a preferred source' button: eligibility check, a button styled to the site using Google's official code, placement after the best paragraph, and a live verify. Readers who choose the site see it more in Top Stories and get a 'preferred' badge in AI Overviews and AI Mode.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>/mos-geo-google-preferred-sources</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>campaigns/geo/YYYY-MM/preferred-sources/</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Initiatives</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="n"/>
       <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-dealbreakers: Client website URL (community or marketplace URLs optional); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+; mos-geo-fan-out-map: Gemini API key (free tier); mos-geo-google-preferred-sources: Client website URL (site code or WordPress access to install; otherwise a developer handover)</t>
-        </is>
-      </c>
+      <c r="B18" s="4" t="n"/>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
@@ -1040,7 +1068,11 @@
       <c r="K18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="n"/>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Needs: mos-geo-brand-360: DataForSEO (OpenRouter, Bright Data optional); mos-geo-ai-info: Client website URL (uses Brand Truth Review corrections when present); mos-geo-dealbreakers: Client website URL (community or marketplace URLs optional); mos-geo-review-sentiment: Apify token (about $0.50 to $3 a run at 500 reviews per platform); TypeSafe API key optional (Claude labels in session without it); mos-geo-llm-buttons: Client website URL; mos-geo-internal-links: Screaming Frog Internal HTML + All Inlinks exports and stored HTML (GSC columns optional); TypeSafe API key for judge/place; mos-geo-schema-scraper: Screaming Frog crawl with JavaScript rendering and a JSON-LD custom extraction (or stored HTML); Apify token only for the paid fallback; mos-geo-schema-optimisation: Screaming Frog structured data export (CSV), ideally from the same crawl as the scraper; Node 18+; mos-geo-fan-out-map: Gemini API key (free tier); mos-geo-google-preferred-sources: Client website URL (site code or WordPress access to install; otherwise a developer handover)</t>
+        </is>
+      </c>
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
@@ -1652,6 +1684,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>